<commit_message>
add LCSC partnumber to generic parts
</commit_message>
<xml_diff>
--- a/Project Outputs for uz_per_voltage_card_breakout/Rev01/BOM/BOM_JLC-uz_per_voltage_card_breakout.xlsx
+++ b/Project Outputs for uz_per_voltage_card_breakout/Rev01/BOM/BOM_JLC-uz_per_voltage_card_breakout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\uz_per_voltage_card_breakout\Project Outputs for uz_per_voltage_card_breakout\Rev01\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A669D49-35EE-45AE-825A-3378BB486024}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{331F73A3-9D04-402C-9AB8-8CAF13CFAE58}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="9945" windowHeight="13710" xr2:uid="{145671D1-4D89-4A06-A4E9-64B2107842E9}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="38">
   <si>
     <t>Quantity</t>
   </si>
@@ -136,6 +136,12 @@
   </si>
   <si>
     <t>C492405</t>
+  </si>
+  <si>
+    <t>C2884019</t>
+  </si>
+  <si>
+    <t>C780055</t>
   </si>
 </sst>
 </file>
@@ -524,7 +530,8 @@
     <col min="7" max="7" width="24.7109375" customWidth="1"/>
     <col min="8" max="8" width="8.85546875" customWidth="1"/>
     <col min="9" max="9" width="10.140625" customWidth="1"/>
-    <col min="10" max="11" width="16.7109375" customWidth="1"/>
+    <col min="10" max="10" width="44.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -589,7 +596,9 @@
       <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
@@ -645,7 +654,9 @@
       <c r="J4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="1"/>
+      <c r="K4" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">

</xml_diff>